<commit_message>
NICA: Excel con título de cada video, audiencia, copy por red, simulación, nota y guion por partes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XHpWW3cNoPrwBL8CwPdgsU
</commit_message>
<xml_diff>
--- a/nica-apify/calendario/calendario-semana-2026-10-06.xlsx
+++ b/nica-apify/calendario/calendario-semana-2026-10-06.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet name="Cómo leer" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Calendario" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mi semana" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Podcast y YouTube" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Querido Ex" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Guion por partes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mi semana" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Podcast y YouTube" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Querido Ex" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calendario'!$A$1:$Y$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calendario'!$A$1:$AH$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -567,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -590,115 +591,127 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Una fila = una pieza (18). El mismo video va a las 4 redes de la columna PLATAFORMAS.</t>
+          <t>Una fila = una pieza (18). TÍTULO DEL VIDEO es el nombre de cada pieza. El mismo video va a las 4 redes de la columna PLATAFORMAS. Ahí está todo lo del guion: audiencia, copy de cada red, simulación y nota.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Guion completo por tiempos</t>
+          <t>Guion por partes</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Todo lo que dices, con el segundo en que va cada parte: GANCHO → GUARDAR Y COMPARTIR → DOLOR → HACKEO → REVELACIÓN → COMENTA → CTA. Los tiempos se calculan a ritmo cómodo (unas 150 palabras por minuto) más 6 segundos para que hagan el hackeo contigo.</t>
+          <t>El guion original separado en sus 8 partes (HOOK, GUARDA, PROBLEMA Y SÍNTOMA, REENCUADRE, PUENTE, MICROHERRAMIENTA, REVELACIÓN, CTA), por si quieres verlo así.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Hora (Monterrey)</t>
+          <t>Guion completo por tiempos</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Sale de tus 40 TikToks: de 18 a 21 h rinden 6.3x tu mediana (7 videos) y de 10 a 13 h, 1.6x (5 videos). De 22 a 5 h, donde más publicas (14 videos), rinden 0.5x. Son pocos videos: es una señal, no una certeza. Instagram, Facebook y YouTube no tienen dato propio todavía.</t>
+          <t>Todo lo que dices, con el segundo en que va cada parte: GANCHO → GUARDAR Y COMPARTIR → DOLOR → HACKEO → REVELACIÓN → COMENTA → CTA. Los tiempos se calculan a ritmo cómodo (unas 150 palabras por minuto) más 6 segundos para que hagan el hackeo contigo.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Copy out</t>
+          <t>Hora (Monterrey)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>El texto que pegas al publicar en TikTok, Instagram y Facebook, ya con hashtags. YouTube Shorts lleva su título aparte.</t>
+          <t>Sale de tus 40 TikToks: de 18 a 21 h rinden 6.3x tu mediana (7 videos) y de 10 a 13 h, 1.6x (5 videos). De 22 a 5 h, donde más publicas (14 videos), rinden 0.5x. Son pocos videos: es una señal, no una certeza. Instagram, Facebook y YouTube no tienen dato propio todavía.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Hashtags</t>
+          <t>Copy out</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5 por pieza: #mabradiante + 2 del problema + 1 de tu nicho + #mty (para ser la referente en Monterrey y México). Quitamos #teamwork, #following y #bdtiktokofficial: no tienen relación con tu tema.</t>
+          <t>El texto que pegas al publicar en TikTok, Instagram y Facebook, ya con hashtags. YouTube Shorts lleva su título aparte.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Emoción</t>
+          <t>Hashtags</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>La emoción que busca el gancho: sorpresa, alivio, identificación o curiosidad.</t>
+          <t>5 por pieza: #mabradiante + 2 del problema + 1 de tu nicho + #mty (para ser la referente en Monterrey y México). Quitamos #teamwork, #following y #bdtiktokofficial: no tienen relación con tu tema.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Rendimiento esperado</t>
+          <t>Emoción</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>La meta de cada pieza contra tus propios números. No es una predicción: es la vara para medir.</t>
+          <t>La emoción que busca el gancho: sorpresa, alivio, identificación o curiosidad.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Patrón</t>
+          <t>Rendimiento esperado</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Qué fórmula viral usa la pieza. En la rutina semanal vemos cuál te funcionó y repetimos esa.</t>
+          <t>La meta de cada pieza contra tus propios números. No es una predicción: es la vara para medir.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Celdas amarillas</t>
+          <t>Patrón</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Las llenas tú: ¿Grabado?, ¿Publicado? y tus números reales.</t>
+          <t>Qué fórmula viral usa la pieza. En la rutina semanal vemos cuál te funcionó y repetimos esa.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Celdas amarillas</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Las llenas tú: ¿Grabado?, ¿Publicado?, tus números reales y si coincidió con la simulación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Pestañas</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Calendario · Mi semana · Podcast y YouTube · Querido Ex (los 8 audios completos para leer y grabar).</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Calendario · Guion por partes · Mi semana · Podcast y YouTube · Querido Ex (los 8 audios completos para leer y grabar).</t>
         </is>
       </c>
     </row>
@@ -713,34 +726,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:AH22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="80" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="36" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="36" customWidth="1" min="18" max="18"/>
-    <col width="42" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="80" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="36" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="36" customWidth="1" min="23" max="23"/>
+    <col width="42" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="11" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -761,112 +783,157 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>PIEZA</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>TÍTULO DEL VIDEO</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Nombre interno</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>PLATAFORMAS</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>PIEZA</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>TEMA (problema)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Audiencia</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>TIPO DE HOOK</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>EMOCIÓN</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>GUION COMPLETO POR TIEMPOS (lo que dices)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>DURACIÓN</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>FORMATO</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>CTA: comenta…</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>COPY OUT (TikTok, Instagram y Facebook)</t>
-        </is>
-      </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>COPY OUT · TikTok</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>COPY OUT · Instagram Reels</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>COPY OUT · Facebook Reels</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>Título YouTube Shorts</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>HASHTAGS</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>RENDIMIENTO ESPERADO</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>PATRÓN viral que usa</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>Por qué en este orden y a esta hora</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
-        <is>
-          <t>Calificación vs patrones</t>
-        </is>
-      </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>Simulación (calificación vs patrones, no predice vistas)</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>Nota de la pieza</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>¿Grabado?</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>¿Publicado?</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>Vistas reales</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
+        <is>
+          <t>Likes reales</t>
+        </is>
+      </c>
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>Comentarios reales</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>Compartidos reales</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>¿Coincidió con la simulación?</t>
         </is>
       </c>
     </row>
@@ -883,35 +950,50 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>12:30 (ya pasó: ver pendiente)</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>MAR-1</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>No era ansiedad: era una mente sin dirección</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Martes 06 · Pieza 1 · Ansiedad · mente que no para</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>MAR-1</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Ansiedad · mente que no para</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>A y B</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>G1 · Confesión + reencuadre</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>[0:00–0:07] GANCHO: "Durante años creí que tenía ansiedad. Lo que tenía era una mente que nadie me enseñó a dirigir."
 [0:07–0:14] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien cuya mente no se apaga."
@@ -922,67 +1004,99 @@
 [1:09–1:13] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>≈ 1:13 min (73 s)</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>MENTE</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>Durante años creí que tenía ansiedad… 🧠 Guarda este video y compártelo con alguien cuya mente no para. Comenta MENTE 👇
 #mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Durante años creí que tenía ansiedad… 🧠 Guarda este video y compártelo con alguien cuya mente no para. Comenta MENTE 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Durante años creí que tenía ansiedad… 🧠 Guarda este video y compártelo con alguien cuya mente no para. Comenta MENTE 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
         <is>
           <t>No era ansiedad: era una mente sin dirección #mabradiante #ansiedad #calmamental #hackeatumente #mty #shorts</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="U2" s="5" t="inlineStr">
         <is>
           <t>#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr">
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="X2" s="5" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T2" s="5" t="inlineStr">
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr"/>
-      <c r="V2" s="7" t="inlineStr"/>
-      <c r="W2" s="7" t="inlineStr"/>
-      <c r="X2" s="7" t="inlineStr"/>
-      <c r="Y2" s="7" t="inlineStr"/>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>Pieza de historia personal (TDAH): sin venta.</t>
+        </is>
+      </c>
+      <c r="AB2" s="7" t="inlineStr"/>
+      <c r="AC2" s="7" t="inlineStr"/>
+      <c r="AD2" s="7" t="inlineStr"/>
+      <c r="AE2" s="7" t="inlineStr"/>
+      <c r="AF2" s="7" t="inlineStr"/>
+      <c r="AG2" s="7" t="inlineStr"/>
+      <c r="AH2" s="7" t="inlineStr"/>
     </row>
     <row r="3" ht="330" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -997,35 +1111,50 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>18:30 (ya pasó: ver pendiente)</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>MAR-2</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Respiración de 60 segundos para la ansiedad</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Martes 06 · Pieza 2 · Ansiedad · ataque en el cuerpo</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>MAR-2</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Ansiedad · ataque en el cuerpo</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>G2 · Promesa práctica</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Alivio: "algo que puedo hacer ya"</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>[0:00–0:05] GANCHO: "Haz esto 60 segundos cuando sientas que la ansiedad te sube al pecho."
 [0:05–0:12] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien cuya mente no se apaga."
@@ -1036,67 +1165,99 @@
 [1:03–1:07] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>≈ 1:07 min (67 s)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>CALMA</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>60 segundos para bajar la ansiedad desde el cuerpo 🫁 Guárdalo antes de que se te pierda. Comenta CALMA 👇
 #mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>60 segundos para bajar la ansiedad desde el cuerpo 🫁 Guárdalo antes de que se te pierda. Comenta CALMA 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>60 segundos para bajar la ansiedad desde el cuerpo 🫁 Guárdalo antes de que se te pierda. Comenta CALMA 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>Respiración de 60 segundos para la ansiedad #mabradiante #ansiedad #calmamental #hackeatumente #mty #shorts</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>Algo para usar ya: decreto, respiración o ritual (tu viral de 2.2M y tus 4 más vistos)</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="X3" s="5" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U3" s="7" t="inlineStr"/>
-      <c r="V3" s="7" t="inlineStr"/>
-      <c r="W3" s="7" t="inlineStr"/>
-      <c r="X3" s="7" t="inlineStr"/>
-      <c r="Y3" s="7" t="inlineStr"/>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="inlineStr"/>
+      <c r="AC3" s="7" t="inlineStr"/>
+      <c r="AD3" s="7" t="inlineStr"/>
+      <c r="AE3" s="7" t="inlineStr"/>
+      <c r="AF3" s="7" t="inlineStr"/>
+      <c r="AG3" s="7" t="inlineStr"/>
+      <c r="AH3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="330" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -1111,35 +1272,50 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>20:30 (ya pasó: ver pendiente)</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>MAR-3</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Por qué tu mente se acelera al dormir</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Martes 06 · Pieza 3 · Ansiedad · insomnio</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>MAR-3</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Ansiedad · insomnio</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>A y B</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>G4 · Pregunta-dolor</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Identificación: "eso me pasa a mí"</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>[0:00–0:06] GANCHO: "¿Por qué tu mente se acelera justo cuando por fin te acuestas a dormir?"
 [0:06–0:13] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien cuya mente no se apaga."
@@ -1150,67 +1326,99 @@
 [1:03–1:12] CTA: "Si tu mente no te deja dormir, en Querida Ansiedad te doy la auditoría mental y los audios para bajar su velocidad."</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>≈ 1:12 min (72 s)</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>DORMIR</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Querida Ansiedad · $399</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>¿Tu mente se prende justo cuando te acuestas? 🌙 Guarda este hackeo para esta noche. Comenta DORMIR 👇
 #mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>¿Tu mente se prende justo cuando te acuestas? 🌙 Guarda este hackeo para esta noche. Comenta DORMIR 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>¿Tu mente se prende justo cuando te acuestas? 🌙 Guarda este hackeo para esta noche. Comenta DORMIR 👇
+#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>Por qué tu mente se acelera al dormir #mabradiante #ansiedad #calmamental #hackeatumente #mty #shorts</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>#mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr">
         <is>
           <t>Pregunta-dolor: nombrar lo que ella siente en sus palabras</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="X4" s="5" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U4" s="7" t="inlineStr"/>
-      <c r="V4" s="7" t="inlineStr"/>
-      <c r="W4" s="7" t="inlineStr"/>
-      <c r="X4" s="7" t="inlineStr"/>
-      <c r="Y4" s="7" t="inlineStr"/>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>Pieza de venta del día (1 de 3).</t>
+        </is>
+      </c>
+      <c r="AB4" s="7" t="inlineStr"/>
+      <c r="AC4" s="7" t="inlineStr"/>
+      <c r="AD4" s="7" t="inlineStr"/>
+      <c r="AE4" s="7" t="inlineStr"/>
+      <c r="AF4" s="7" t="inlineStr"/>
+      <c r="AG4" s="7" t="inlineStr"/>
+      <c r="AH4" s="7" t="inlineStr"/>
     </row>
     <row r="5" ht="330" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1228,32 +1436,47 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-1</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Por qué repites la misma relación</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Miércoles 07 · Pieza 1 · Relaciones · repetir la misma historia</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>MIÉ-1</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Relaciones · repetir la misma historia</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>G1 · Reencuadre</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>[0:00–0:08] GANCHO: "No es que siempre te toque la persona equivocada. Es que tu sistema reconoce como 'amor' lo que ya conoce."
 [0:08–0:17] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con esa amiga que siempre repite la misma historia en el amor."
@@ -1264,67 +1487,99 @@
 [1:06–1:10] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>≈ 1:10 min (70 s)</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>PATRÓN</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr">
+      <c r="Q5" s="8" t="inlineStr">
         <is>
           <t>¿Siempre te toca la persona equivocada? 💔 Guárdalo y compártelo con tu amiga que repite la historia. Comenta PATRÓN 👇
 #mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>¿Siempre te toca la persona equivocada? 💔 Guárdalo y compártelo con tu amiga que repite la historia. Comenta PATRÓN 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>¿Siempre te toca la persona equivocada? 💔 Guárdalo y compártelo con tu amiga que repite la historia. Comenta PATRÓN 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
         <is>
           <t>Por qué repites la misma relación #mabradiante #relaciones #amorpropio #dependenciaemocional #mty #shorts</t>
         </is>
       </c>
-      <c r="P5" s="8" t="inlineStr">
+      <c r="U5" s="8" t="inlineStr">
         <is>
           <t>#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="Q5" s="8" t="inlineStr">
+      <c r="V5" s="8" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="W5" s="8" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S5" s="8" t="inlineStr">
+      <c r="X5" s="8" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T5" s="8" t="inlineStr">
+      <c r="Y5" s="8" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z5" s="8" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U5" s="7" t="inlineStr"/>
-      <c r="V5" s="7" t="inlineStr"/>
-      <c r="W5" s="7" t="inlineStr"/>
-      <c r="X5" s="7" t="inlineStr"/>
-      <c r="Y5" s="7" t="inlineStr"/>
+      <c r="AA5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB5" s="7" t="inlineStr"/>
+      <c r="AC5" s="7" t="inlineStr"/>
+      <c r="AD5" s="7" t="inlineStr"/>
+      <c r="AE5" s="7" t="inlineStr"/>
+      <c r="AF5" s="7" t="inlineStr"/>
+      <c r="AG5" s="7" t="inlineStr"/>
+      <c r="AH5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="330" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1342,32 +1597,47 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-2</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Di esto antes de escribirle</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Miércoles 07 · Pieza 2 · Relaciones · apego</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>MIÉ-2</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Relaciones · apego</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>G2 · Promesa práctica</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>Alivio: "algo que puedo hacer ya"</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>[0:00–0:04] GANCHO: "Di esto antes de volver a escribirle a esa persona."
 [0:04–0:13] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con esa amiga que siempre repite la misma historia en el amor."
@@ -1378,67 +1648,99 @@
 [1:05–1:09] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>≈ 1:09 min (69 s)</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>ME ELIJO</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr">
+      <c r="Q6" s="8" t="inlineStr">
         <is>
           <t>Antes de escribirle otra vez, di esto 📵💜 Guárdalo para cuando lo necesites. Comenta ME ELIJO 👇
 #mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="O6" s="8" t="inlineStr">
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>Antes de escribirle otra vez, di esto 📵💜 Guárdalo para cuando lo necesites. Comenta ME ELIJO 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>Antes de escribirle otra vez, di esto 📵💜 Guárdalo para cuando lo necesites. Comenta ME ELIJO 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="T6" s="8" t="inlineStr">
         <is>
           <t>Di esto antes de escribirle #mabradiante #relaciones #amorpropio #dependenciaemocional #mty #shorts</t>
         </is>
       </c>
-      <c r="P6" s="8" t="inlineStr">
+      <c r="U6" s="8" t="inlineStr">
         <is>
           <t>#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="Q6" s="8" t="inlineStr">
+      <c r="V6" s="8" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R6" s="8" t="inlineStr">
+      <c r="W6" s="8" t="inlineStr">
         <is>
           <t>Algo para usar ya: decreto, respiración o ritual (tu viral de 2.2M y tus 4 más vistos)</t>
         </is>
       </c>
-      <c r="S6" s="8" t="inlineStr">
+      <c r="X6" s="8" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T6" s="8" t="inlineStr">
+      <c r="Y6" s="8" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z6" s="8" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U6" s="7" t="inlineStr"/>
-      <c r="V6" s="7" t="inlineStr"/>
-      <c r="W6" s="7" t="inlineStr"/>
-      <c r="X6" s="7" t="inlineStr"/>
-      <c r="Y6" s="7" t="inlineStr"/>
+      <c r="AA6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB6" s="7" t="inlineStr"/>
+      <c r="AC6" s="7" t="inlineStr"/>
+      <c r="AD6" s="7" t="inlineStr"/>
+      <c r="AE6" s="7" t="inlineStr"/>
+      <c r="AF6" s="7" t="inlineStr"/>
+      <c r="AG6" s="7" t="inlineStr"/>
+      <c r="AH6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="330" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -1456,32 +1758,47 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-3</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Deja de esperar a que te elijan</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Miércoles 07 · Pieza 3 · Relaciones · necesitar que te elijan</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>MIÉ-3</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>Relaciones · necesitar que te elijan</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>A y B</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>G4 · Pregunta-dolor</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>Identificación: "eso me pasa a mí"</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="L7" s="8" t="inlineStr">
         <is>
           <t>[0:00–0:05] GANCHO: "Si sigues esperando a que alguien te elija, este video es para ti."
 [0:05–0:14] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con esa amiga que siempre repite la misma historia en el amor."
@@ -1492,67 +1809,99 @@
 [1:00–1:06] CTA: "En Crea y Activa tu Alter Ego te guío paso a paso para instalar esa identidad."</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>≈ 1:06 min (66 s)</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>ALTER EGO</t>
         </is>
       </c>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="P7" s="8" t="inlineStr">
         <is>
           <t>Crea y Activa tu Alter Ego · $599</t>
         </is>
       </c>
-      <c r="N7" s="8" t="inlineStr">
+      <c r="Q7" s="8" t="inlineStr">
         <is>
           <t>Deja de esperar a que te elijan ✨ Guarda este ejercicio de 7 días. Comenta ALTER EGO 👇
 #mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="O7" s="8" t="inlineStr">
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>Deja de esperar a que te elijan ✨ Guarda este ejercicio de 7 días. Comenta ALTER EGO 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>Deja de esperar a que te elijan ✨ Guarda este ejercicio de 7 días. Comenta ALTER EGO 👇
+#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
         <is>
           <t>Deja de esperar a que te elijan #mabradiante #relaciones #amorpropio #dependenciaemocional #mty #shorts</t>
         </is>
       </c>
-      <c r="P7" s="8" t="inlineStr">
+      <c r="U7" s="8" t="inlineStr">
         <is>
           <t>#mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
-      <c r="Q7" s="8" t="inlineStr">
+      <c r="V7" s="8" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R7" s="8" t="inlineStr">
+      <c r="W7" s="8" t="inlineStr">
         <is>
           <t>Pregunta-dolor: nombrar lo que ella siente en sus palabras</t>
         </is>
       </c>
-      <c r="S7" s="8" t="inlineStr">
+      <c r="X7" s="8" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T7" s="8" t="inlineStr">
+      <c r="Y7" s="8" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z7" s="8" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U7" s="7" t="inlineStr"/>
-      <c r="V7" s="7" t="inlineStr"/>
-      <c r="W7" s="7" t="inlineStr"/>
-      <c r="X7" s="7" t="inlineStr"/>
-      <c r="Y7" s="7" t="inlineStr"/>
+      <c r="AA7" s="8" t="inlineStr">
+        <is>
+          <t>Pieza de venta del día (1 de 3).</t>
+        </is>
+      </c>
+      <c r="AB7" s="7" t="inlineStr"/>
+      <c r="AC7" s="7" t="inlineStr"/>
+      <c r="AD7" s="7" t="inlineStr"/>
+      <c r="AE7" s="7" t="inlineStr"/>
+      <c r="AF7" s="7" t="inlineStr"/>
+      <c r="AG7" s="7" t="inlineStr"/>
+      <c r="AH7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="330" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
@@ -1570,32 +1919,47 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>JUE-1</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>No estás perdida: estás despertando</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Jueves 08 · Pieza 1 · Vacío · la vida ya no alcanza</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>JUE-1</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>Vacío · la vida ya no alcanza</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>G4 · Pregunta-dolor</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Identificación: "eso me pasa a mí"</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="L8" s="10" t="inlineStr">
         <is>
           <t>[0:00–0:05] GANCHO: "¿Por qué ya no te hace feliz una vida que antes sí?"
 [0:05–0:12] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que siente que está despertando."
@@ -1606,67 +1970,99 @@
 [0:53–0:57] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="M8" s="10" t="inlineStr">
         <is>
           <t>≈ 0:57 min (57 s)</t>
         </is>
       </c>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="N8" s="10" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="O8" s="10" t="inlineStr">
         <is>
           <t>DESPERTANDO</t>
         </is>
       </c>
-      <c r="M8" s="10" t="inlineStr">
+      <c r="P8" s="10" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="Q8" s="10" t="inlineStr">
         <is>
           <t>¿Y si no estás perdida… estás despertando? 🌀 Guárdalo y compártelo con quien lo necesita. Comenta DESPERTANDO 👇
 #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="O8" s="10" t="inlineStr">
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>¿Y si no estás perdida… estás despertando? 🌀 Guárdalo y compártelo con quien lo necesita. Comenta DESPERTANDO 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="S8" s="10" t="inlineStr">
+        <is>
+          <t>¿Y si no estás perdida… estás despertando? 🌀 Guárdalo y compártelo con quien lo necesita. Comenta DESPERTANDO 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="T8" s="10" t="inlineStr">
         <is>
           <t>No estás perdida: estás despertando #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty #shorts</t>
         </is>
       </c>
-      <c r="P8" s="10" t="inlineStr">
+      <c r="U8" s="10" t="inlineStr">
         <is>
           <t>#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="Q8" s="10" t="inlineStr">
+      <c r="V8" s="10" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R8" s="10" t="inlineStr">
+      <c r="W8" s="10" t="inlineStr">
         <is>
           <t>Pregunta-dolor: nombrar lo que ella siente en sus palabras</t>
         </is>
       </c>
-      <c r="S8" s="10" t="inlineStr">
+      <c r="X8" s="10" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T8" s="10" t="inlineStr">
+      <c r="Y8" s="10" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z8" s="10" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U8" s="7" t="inlineStr"/>
-      <c r="V8" s="7" t="inlineStr"/>
-      <c r="W8" s="7" t="inlineStr"/>
-      <c r="X8" s="7" t="inlineStr"/>
-      <c r="Y8" s="7" t="inlineStr"/>
+      <c r="AA8" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB8" s="7" t="inlineStr"/>
+      <c r="AC8" s="7" t="inlineStr"/>
+      <c r="AD8" s="7" t="inlineStr"/>
+      <c r="AE8" s="7" t="inlineStr"/>
+      <c r="AF8" s="7" t="inlineStr"/>
+      <c r="AG8" s="7" t="inlineStr"/>
+      <c r="AH8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="330" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -1684,32 +2080,47 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>JUE-2</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>200 herramientas y ningún sistema</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Jueves 08 · Pieza 2 · Vacío · información sin sistema (audiencia avanzada)</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>JUE-2</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>Vacío · información sin sistema (audiencia avanzada)</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>G1 · Reencuadre</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="L9" s="10" t="inlineStr">
         <is>
           <t>[0:00–0:06] GANCHO: "Si sabes de energía, chakras, neuro y biohacking, pero sientes que todo está desconectado, escucha esto."
 [0:06–0:13] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que siente que está despertando."
@@ -1720,67 +2131,99 @@
 [1:04–1:08] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="M9" s="10" t="inlineStr">
         <is>
           <t>≈ 1:08 min (68 s)</t>
         </is>
       </c>
-      <c r="K9" s="10" t="inlineStr">
+      <c r="N9" s="10" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L9" s="10" t="inlineStr">
+      <c r="O9" s="10" t="inlineStr">
         <is>
           <t>MAPA</t>
         </is>
       </c>
-      <c r="M9" s="10" t="inlineStr">
+      <c r="P9" s="10" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N9" s="10" t="inlineStr">
+      <c r="Q9" s="10" t="inlineStr">
         <is>
           <t>Tienes demasiada información y muy poco sistema 🗺️ Guárdalo. Comenta MAPA 👇
 #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="O9" s="10" t="inlineStr">
+      <c r="R9" s="10" t="inlineStr">
+        <is>
+          <t>Tienes demasiada información y muy poco sistema 🗺️ Guárdalo. Comenta MAPA 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>Tienes demasiada información y muy poco sistema 🗺️ Guárdalo. Comenta MAPA 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="T9" s="10" t="inlineStr">
         <is>
           <t>200 herramientas y ningún sistema #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty #shorts</t>
         </is>
       </c>
-      <c r="P9" s="10" t="inlineStr">
+      <c r="U9" s="10" t="inlineStr">
         <is>
           <t>#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="Q9" s="10" t="inlineStr">
+      <c r="V9" s="10" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R9" s="10" t="inlineStr">
+      <c r="W9" s="10" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S9" s="10" t="inlineStr">
+      <c r="X9" s="10" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T9" s="10" t="inlineStr">
+      <c r="Y9" s="10" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z9" s="10" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U9" s="7" t="inlineStr"/>
-      <c r="V9" s="7" t="inlineStr"/>
-      <c r="W9" s="7" t="inlineStr"/>
-      <c r="X9" s="7" t="inlineStr"/>
-      <c r="Y9" s="7" t="inlineStr"/>
+      <c r="AA9" s="10" t="inlineStr">
+        <is>
+          <t>Siembra BNQ™ para la audiencia avanzada, sin vender.</t>
+        </is>
+      </c>
+      <c r="AB9" s="7" t="inlineStr"/>
+      <c r="AC9" s="7" t="inlineStr"/>
+      <c r="AD9" s="7" t="inlineStr"/>
+      <c r="AE9" s="7" t="inlineStr"/>
+      <c r="AF9" s="7" t="inlineStr"/>
+      <c r="AG9" s="7" t="inlineStr"/>
+      <c r="AH9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="330" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -1798,32 +2241,47 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>JUE-3</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>7 señales de que estás despertando</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Jueves 08 · Pieza 3 · Vacío · quiero despertar y no sé cómo</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>JUE-3</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Vacío · quiero despertar y no sé cómo</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>G5 · Espejo/lista</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Curiosidad: "¿me pasa a mí?"</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>[0:00–0:05] GANCHO: "La primera señal de un despertar no es sentir paz. Es sentir incomodidad."
 [0:05–0:12] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que siente que está despertando."
@@ -1834,67 +2292,99 @@
 [0:54–0:57] CTA: "Hice DESPIERTA para darte ese primer mapa."</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
         <is>
           <t>≈ 0:57 min (57 s)</t>
         </is>
       </c>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="N10" s="10" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="O10" s="10" t="inlineStr">
         <is>
           <t>DESPIERTA</t>
         </is>
       </c>
-      <c r="M10" s="10" t="inlineStr">
+      <c r="P10" s="10" t="inlineStr">
         <is>
           <t>DESPIERTA · $499</t>
         </is>
       </c>
-      <c r="N10" s="10" t="inlineStr">
+      <c r="Q10" s="10" t="inlineStr">
         <is>
           <t>7 señales de que estás despertando y nadie te lo explicó 🌀 Guarda la lista. Comenta DESPIERTA 👇
 #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="O10" s="10" t="inlineStr">
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t>7 señales de que estás despertando y nadie te lo explicó 🌀 Guarda la lista. Comenta DESPIERTA 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>7 señales de que estás despertando y nadie te lo explicó 🌀 Guarda la lista. Comenta DESPIERTA 👇
+#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
+        </is>
+      </c>
+      <c r="T10" s="10" t="inlineStr">
         <is>
           <t>7 señales de que estás despertando #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty #shorts</t>
         </is>
       </c>
-      <c r="P10" s="10" t="inlineStr">
+      <c r="U10" s="10" t="inlineStr">
         <is>
           <t>#mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
-      <c r="Q10" s="10" t="inlineStr">
+      <c r="V10" s="10" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R10" s="10" t="inlineStr">
+      <c r="W10" s="10" t="inlineStr">
         <is>
           <t>Lista o espejo: "señales de que…" (formato lista que se guarda)</t>
         </is>
       </c>
-      <c r="S10" s="10" t="inlineStr">
+      <c r="X10" s="10" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T10" s="10" t="inlineStr">
+      <c r="Y10" s="10" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 1/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 9/10</t>
+        </is>
+      </c>
+      <c r="Z10" s="10" t="inlineStr">
         <is>
           <t>9/10</t>
         </is>
       </c>
-      <c r="U10" s="7" t="inlineStr"/>
-      <c r="V10" s="7" t="inlineStr"/>
-      <c r="W10" s="7" t="inlineStr"/>
-      <c r="X10" s="7" t="inlineStr"/>
-      <c r="Y10" s="7" t="inlineStr"/>
+      <c r="AA10" s="10" t="inlineStr">
+        <is>
+          <t>Pieza de venta del día (1 de 3). El gancho es tipo lista (G5): vale 1 de 2.</t>
+        </is>
+      </c>
+      <c r="AB10" s="7" t="inlineStr"/>
+      <c r="AC10" s="7" t="inlineStr"/>
+      <c r="AD10" s="7" t="inlineStr"/>
+      <c r="AE10" s="7" t="inlineStr"/>
+      <c r="AF10" s="7" t="inlineStr"/>
+      <c r="AG10" s="7" t="inlineStr"/>
+      <c r="AH10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="330" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
@@ -1912,32 +2402,47 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>VIE-1</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>No estás cansada: estás en alerta</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Viernes 09 · Pieza 1 · Cansancio · siempre agotada</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>VIE-1</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Cansancio · siempre agotada</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>G1 · Reencuadre</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="L11" s="12" t="inlineStr">
         <is>
           <t>[0:00–0:08] GANCHO: "No estás cansada por todo lo que haces. Estás cansada por todo lo que tu cuerpo carga en alerta."
 [0:08–0:17] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -1948,67 +2453,99 @@
 [0:59–1:03] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="M11" s="12" t="inlineStr">
         <is>
           <t>≈ 1:03 min (63 s)</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
+      <c r="N11" s="12" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L11" s="12" t="inlineStr">
+      <c r="O11" s="12" t="inlineStr">
         <is>
           <t>ENERGÍA</t>
         </is>
       </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N11" s="12" t="inlineStr">
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>No es flojera: es tu cuerpo en alerta 🔋 Guarda este escaneo de 30 segundos. Comenta ENERGÍA 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O11" s="12" t="inlineStr">
+      <c r="R11" s="12" t="inlineStr">
+        <is>
+          <t>No es flojera: es tu cuerpo en alerta 🔋 Guarda este escaneo de 30 segundos. Comenta ENERGÍA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S11" s="12" t="inlineStr">
+        <is>
+          <t>No es flojera: es tu cuerpo en alerta 🔋 Guarda este escaneo de 30 segundos. Comenta ENERGÍA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T11" s="12" t="inlineStr">
         <is>
           <t>No estás cansada: estás en alerta #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P11" s="12" t="inlineStr">
+      <c r="U11" s="12" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr">
+      <c r="V11" s="12" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R11" s="12" t="inlineStr">
+      <c r="W11" s="12" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S11" s="12" t="inlineStr">
+      <c r="X11" s="12" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T11" s="12" t="inlineStr">
+      <c r="Y11" s="12" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z11" s="12" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U11" s="7" t="inlineStr"/>
-      <c r="V11" s="7" t="inlineStr"/>
-      <c r="W11" s="7" t="inlineStr"/>
-      <c r="X11" s="7" t="inlineStr"/>
-      <c r="Y11" s="7" t="inlineStr"/>
+      <c r="AA11" s="12" t="inlineStr">
+        <is>
+          <t>Sin promesas de salud: si el cansancio es fuerte o constante, recomendar ir al médico.</t>
+        </is>
+      </c>
+      <c r="AB11" s="7" t="inlineStr"/>
+      <c r="AC11" s="7" t="inlineStr"/>
+      <c r="AD11" s="7" t="inlineStr"/>
+      <c r="AE11" s="7" t="inlineStr"/>
+      <c r="AF11" s="7" t="inlineStr"/>
+      <c r="AG11" s="7" t="inlineStr"/>
+      <c r="AH11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="330" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
@@ -2026,32 +2563,47 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>VIE-2</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Haz esto antes de tocar el celular</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Viernes 09 · Pieza 2 · Energía · arrancar el día en caos</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>VIE-2</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Energía · arrancar el día en caos</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>G2 · Promesa práctica</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="K12" s="12" t="inlineStr">
         <is>
           <t>Alivio: "algo que puedo hacer ya"</t>
         </is>
       </c>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="L12" s="12" t="inlineStr">
         <is>
           <t>[0:00–0:07] GANCHO: "Haz esto al despertar, antes de tocar el celular, y vas a sentir la diferencia en tu energía."
 [0:07–0:14] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que vive cansada aunque duerma."
@@ -2062,67 +2614,99 @@
 [1:03–1:07] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="M12" s="12" t="inlineStr">
         <is>
           <t>≈ 1:07 min (67 s)</t>
         </is>
       </c>
-      <c r="K12" s="12" t="inlineStr">
+      <c r="N12" s="12" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L12" s="12" t="inlineStr">
+      <c r="O12" s="12" t="inlineStr">
         <is>
           <t>SOBERANA</t>
         </is>
       </c>
-      <c r="M12" s="12" t="inlineStr">
+      <c r="P12" s="12" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N12" s="12" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>El minuto que cambia tu energía antes del celular ☀️ Guárdalo para mañana. Comenta SOBERANA 👇
 #mabradiante #energia #modosupervivencia #ritual #mty</t>
         </is>
       </c>
-      <c r="O12" s="12" t="inlineStr">
+      <c r="R12" s="12" t="inlineStr">
+        <is>
+          <t>El minuto que cambia tu energía antes del celular ☀️ Guárdalo para mañana. Comenta SOBERANA 👇
+#mabradiante #energia #modosupervivencia #ritual #mty</t>
+        </is>
+      </c>
+      <c r="S12" s="12" t="inlineStr">
+        <is>
+          <t>El minuto que cambia tu energía antes del celular ☀️ Guárdalo para mañana. Comenta SOBERANA 👇
+#mabradiante #energia #modosupervivencia #ritual #mty</t>
+        </is>
+      </c>
+      <c r="T12" s="12" t="inlineStr">
         <is>
           <t>Haz esto antes de tocar el celular #mabradiante #energia #modosupervivencia #ritual #mty #shorts</t>
         </is>
       </c>
-      <c r="P12" s="12" t="inlineStr">
+      <c r="U12" s="12" t="inlineStr">
         <is>
           <t>#mabradiante #energia #modosupervivencia #ritual #mty</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="V12" s="12" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R12" s="12" t="inlineStr">
+      <c r="W12" s="12" t="inlineStr">
         <is>
           <t>Algo para usar ya: decreto, respiración o ritual (tu viral de 2.2M y tus 4 más vistos)</t>
         </is>
       </c>
-      <c r="S12" s="12" t="inlineStr">
+      <c r="X12" s="12" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T12" s="12" t="inlineStr">
+      <c r="Y12" s="12" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z12" s="12" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U12" s="7" t="inlineStr"/>
-      <c r="V12" s="7" t="inlineStr"/>
-      <c r="W12" s="7" t="inlineStr"/>
-      <c r="X12" s="7" t="inlineStr"/>
-      <c r="Y12" s="7" t="inlineStr"/>
+      <c r="AA12" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB12" s="7" t="inlineStr"/>
+      <c r="AC12" s="7" t="inlineStr"/>
+      <c r="AD12" s="7" t="inlineStr"/>
+      <c r="AE12" s="7" t="inlineStr"/>
+      <c r="AF12" s="7" t="inlineStr"/>
+      <c r="AG12" s="7" t="inlineStr"/>
+      <c r="AH12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="330" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -2140,32 +2724,47 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>VIE-3</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Señales de que vives en modo supervivencia</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Viernes 09 · Pieza 3 · Estrés · modo supervivencia</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>VIE-3</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>Estrés · modo supervivencia</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>A y B</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>G4 · Pregunta-dolor</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="K13" s="12" t="inlineStr">
         <is>
           <t>Identificación: "eso me pasa a mí"</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="L13" s="12" t="inlineStr">
         <is>
           <t>[0:00–0:04] GANCHO: "¿Vives en modo supervivencia y ni siquiera te das cuenta?"
 [0:04–0:13] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -2176,67 +2775,99 @@
 [1:01–1:09] CTA: "En Apaga el Modo Supervivencia tienes el protocolo de biohacking para armonizar tu sistema nervioso y volver al presente."</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="M13" s="12" t="inlineStr">
         <is>
           <t>≈ 1:09 min (69 s)</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
+      <c r="N13" s="12" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
+      <c r="O13" s="12" t="inlineStr">
         <is>
           <t>VUELVO A MÍ</t>
         </is>
       </c>
-      <c r="M13" s="12" t="inlineStr">
+      <c r="P13" s="12" t="inlineStr">
         <is>
           <t>Apaga el Modo Supervivencia · $750</t>
         </is>
       </c>
-      <c r="N13" s="12" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>¿Vives en modo supervivencia? 🧬 Guarda este hackeo de 2 minutos. Comenta VUELVO A MÍ 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O13" s="12" t="inlineStr">
+      <c r="R13" s="12" t="inlineStr">
+        <is>
+          <t>¿Vives en modo supervivencia? 🧬 Guarda este hackeo de 2 minutos. Comenta VUELVO A MÍ 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S13" s="12" t="inlineStr">
+        <is>
+          <t>¿Vives en modo supervivencia? 🧬 Guarda este hackeo de 2 minutos. Comenta VUELVO A MÍ 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T13" s="12" t="inlineStr">
         <is>
           <t>Señales de que vives en modo supervivencia #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P13" s="12" t="inlineStr">
+      <c r="U13" s="12" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="V13" s="12" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R13" s="12" t="inlineStr">
+      <c r="W13" s="12" t="inlineStr">
         <is>
           <t>Pregunta-dolor: nombrar lo que ella siente en sus palabras</t>
         </is>
       </c>
-      <c r="S13" s="12" t="inlineStr">
+      <c r="X13" s="12" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T13" s="12" t="inlineStr">
+      <c r="Y13" s="12" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z13" s="12" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U13" s="7" t="inlineStr"/>
-      <c r="V13" s="7" t="inlineStr"/>
-      <c r="W13" s="7" t="inlineStr"/>
-      <c r="X13" s="7" t="inlineStr"/>
-      <c r="Y13" s="7" t="inlineStr"/>
+      <c r="AA13" s="12" t="inlineStr">
+        <is>
+          <t>Pieza de venta del día (1 de 3). Sin promesas de curación.</t>
+        </is>
+      </c>
+      <c r="AB13" s="7" t="inlineStr"/>
+      <c r="AC13" s="7" t="inlineStr"/>
+      <c r="AD13" s="7" t="inlineStr"/>
+      <c r="AE13" s="7" t="inlineStr"/>
+      <c r="AF13" s="7" t="inlineStr"/>
+      <c r="AG13" s="7" t="inlineStr"/>
+      <c r="AH13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="330" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
@@ -2254,32 +2885,47 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-1</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>La meta que siempre dejas para el próximo año</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Sábado 10 · Pieza 1 · Metas · 'este año sí'</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>SÁB-1</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>Metas · 'este año sí'</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
         <is>
           <t>G4 · Pregunta-dolor</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="K14" s="14" t="inlineStr">
         <is>
           <t>Identificación: "eso me pasa a mí"</t>
         </is>
       </c>
-      <c r="I14" s="14" t="inlineStr">
+      <c r="L14" s="14" t="inlineStr">
         <is>
           <t>[0:00–0:03] GANCHO: "¿Qué meta llevas años diciendo 'este año sí'?"
 [0:03–0:11] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que lleva años diciendo "este año sí"."
@@ -2290,67 +2936,99 @@
 [1:01–1:05] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J14" s="14" t="inlineStr">
+      <c r="M14" s="14" t="inlineStr">
         <is>
           <t>≈ 1:05 min (65 s)</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
+      <c r="N14" s="14" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L14" s="14" t="inlineStr">
+      <c r="O14" s="14" t="inlineStr">
         <is>
           <t>tu meta</t>
         </is>
       </c>
-      <c r="M14" s="14" t="inlineStr">
+      <c r="P14" s="14" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N14" s="14" t="inlineStr">
+      <c r="Q14" s="14" t="inlineStr">
         <is>
           <t>¿Qué meta llevas años diciendo 'este año sí'? 🎯 Escríbela en los comentarios: respondo las que más se repitan.
 #mabradiante #metas #leydeatraccion #decreto #mty</t>
         </is>
       </c>
-      <c r="O14" s="14" t="inlineStr">
+      <c r="R14" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué meta llevas años diciendo 'este año sí'? 🎯 Escríbela en los comentarios: respondo las que más se repitan.
+#mabradiante #metas #leydeatraccion #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S14" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué meta llevas años diciendo 'este año sí'? 🎯 Escríbela en los comentarios: respondo las que más se repitan.
+#mabradiante #metas #leydeatraccion #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T14" s="14" t="inlineStr">
         <is>
           <t>La meta que siempre dejas para el próximo año #mabradiante #metas #leydeatraccion #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P14" s="14" t="inlineStr">
+      <c r="U14" s="14" t="inlineStr">
         <is>
           <t>#mabradiante #metas #leydeatraccion #decreto #mty</t>
         </is>
       </c>
-      <c r="Q14" s="14" t="inlineStr">
+      <c r="V14" s="14" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R14" s="14" t="inlineStr">
+      <c r="W14" s="14" t="inlineStr">
         <is>
           <t>Pregunta-dolor: nombrar lo que ella siente en sus palabras</t>
         </is>
       </c>
-      <c r="S14" s="14" t="inlineStr">
+      <c r="X14" s="14" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T14" s="14" t="inlineStr">
+      <c r="Y14" s="14" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 0/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 9/10</t>
+        </is>
+      </c>
+      <c r="Z14" s="14" t="inlineStr">
         <is>
           <t>9/10</t>
         </is>
       </c>
-      <c r="U14" s="7" t="inlineStr"/>
-      <c r="V14" s="7" t="inlineStr"/>
-      <c r="W14" s="7" t="inlineStr"/>
-      <c r="X14" s="7" t="inlineStr"/>
-      <c r="Y14" s="7" t="inlineStr"/>
+      <c r="AA14" s="14" t="inlineStr">
+        <is>
+          <t>Pieza de comunidad: las respuestas te dan ideas de guiones.</t>
+        </is>
+      </c>
+      <c r="AB14" s="7" t="inlineStr"/>
+      <c r="AC14" s="7" t="inlineStr"/>
+      <c r="AD14" s="7" t="inlineStr"/>
+      <c r="AE14" s="7" t="inlineStr"/>
+      <c r="AF14" s="7" t="inlineStr"/>
+      <c r="AG14" s="7" t="inlineStr"/>
+      <c r="AH14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="330" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
@@ -2368,32 +3046,47 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-2</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>1 minuto para cambiar tu frecuencia</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>Sábado 10 · Pieza 2 · Comunidad · activación juntas</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>SÁB-2</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>Comunidad · activación juntas</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>G2 · Promesa práctica</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
         <is>
           <t>Alivio: "algo que puedo hacer ya"</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr">
+      <c r="L15" s="14" t="inlineStr">
         <is>
           <t>[0:00–0:04] GANCHO: "Hagamos esto juntas ahora: 1 minuto para cambiar tu frecuencia."
 [0:04–0:13] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -2404,67 +3097,99 @@
 [0:56–1:00] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J15" s="14" t="inlineStr">
+      <c r="M15" s="14" t="inlineStr">
         <is>
           <t>≈ 1:00 min (60 s)</t>
         </is>
       </c>
-      <c r="K15" s="14" t="inlineStr">
+      <c r="N15" s="14" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L15" s="14" t="inlineStr">
+      <c r="O15" s="14" t="inlineStr">
         <is>
           <t>COHERENCIA</t>
         </is>
       </c>
-      <c r="M15" s="14" t="inlineStr">
+      <c r="P15" s="14" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N15" s="14" t="inlineStr">
+      <c r="Q15" s="14" t="inlineStr">
         <is>
           <t>1 minuto de coherencia, juntas 💛 Guárdalo y compártelo. Comenta COHERENCIA 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O15" s="14" t="inlineStr">
+      <c r="R15" s="14" t="inlineStr">
+        <is>
+          <t>1 minuto de coherencia, juntas 💛 Guárdalo y compártelo. Comenta COHERENCIA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S15" s="14" t="inlineStr">
+        <is>
+          <t>1 minuto de coherencia, juntas 💛 Guárdalo y compártelo. Comenta COHERENCIA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T15" s="14" t="inlineStr">
         <is>
           <t>1 minuto para cambiar tu frecuencia #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P15" s="14" t="inlineStr">
+      <c r="U15" s="14" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q15" s="14" t="inlineStr">
+      <c r="V15" s="14" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R15" s="14" t="inlineStr">
+      <c r="W15" s="14" t="inlineStr">
         <is>
           <t>Algo para usar ya: decreto, respiración o ritual (tu viral de 2.2M y tus 4 más vistos)</t>
         </is>
       </c>
-      <c r="S15" s="14" t="inlineStr">
+      <c r="X15" s="14" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T15" s="14" t="inlineStr">
+      <c r="Y15" s="14" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z15" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U15" s="7" t="inlineStr"/>
-      <c r="V15" s="7" t="inlineStr"/>
-      <c r="W15" s="7" t="inlineStr"/>
-      <c r="X15" s="7" t="inlineStr"/>
-      <c r="Y15" s="7" t="inlineStr"/>
+      <c r="AA15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB15" s="7" t="inlineStr"/>
+      <c r="AC15" s="7" t="inlineStr"/>
+      <c r="AD15" s="7" t="inlineStr"/>
+      <c r="AE15" s="7" t="inlineStr"/>
+      <c r="AF15" s="7" t="inlineStr"/>
+      <c r="AG15" s="7" t="inlineStr"/>
+      <c r="AH15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="330" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
@@ -2482,32 +3207,47 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-3</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>La creencia que no sabes que tienes</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Sábado 10 · Pieza 3 · Metas · creencias limitantes</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>SÁB-3</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>Metas · creencias limitantes</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>A y B</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>G1 · Creencia rota</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I16" s="14" t="inlineStr">
+      <c r="L16" s="14" t="inlineStr">
         <is>
           <t>[0:00–0:04] GANCHO: "La creencia más peligrosa es la que no sabes que tienes."
 [0:04–0:12] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que lleva años diciendo "este año sí"."
@@ -2518,67 +3258,99 @@
 [0:58–1:06] CTA: "Si quieres hackear la creencia que no te deja avanzar, comenta NIVEL 1 y te mando el link de DESPERTAR."</t>
         </is>
       </c>
-      <c r="J16" s="14" t="inlineStr">
+      <c r="M16" s="14" t="inlineStr">
         <is>
           <t>≈ 1:06 min (66 s)</t>
         </is>
       </c>
-      <c r="K16" s="14" t="inlineStr">
+      <c r="N16" s="14" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L16" s="14" t="inlineStr">
+      <c r="O16" s="14" t="inlineStr">
         <is>
           <t>NIVEL 1</t>
         </is>
       </c>
-      <c r="M16" s="14" t="inlineStr">
+      <c r="P16" s="14" t="inlineStr">
         <is>
           <t>Nivel 1 DESPERTAR · $2,000</t>
         </is>
       </c>
-      <c r="N16" s="14" t="inlineStr">
+      <c r="Q16" s="14" t="inlineStr">
         <is>
           <t>La creencia más peligrosa es la que no sabes que tienes 🔓 Haz el ejercicio. Comenta NIVEL 1 👇
 #mabradiante #metas #leydeatraccion #decreto #mty</t>
         </is>
       </c>
-      <c r="O16" s="14" t="inlineStr">
+      <c r="R16" s="14" t="inlineStr">
+        <is>
+          <t>La creencia más peligrosa es la que no sabes que tienes 🔓 Haz el ejercicio. Comenta NIVEL 1 👇
+#mabradiante #metas #leydeatraccion #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S16" s="14" t="inlineStr">
+        <is>
+          <t>La creencia más peligrosa es la que no sabes que tienes 🔓 Haz el ejercicio. Comenta NIVEL 1 👇
+#mabradiante #metas #leydeatraccion #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T16" s="14" t="inlineStr">
         <is>
           <t>La creencia que no sabes que tienes #mabradiante #metas #leydeatraccion #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P16" s="14" t="inlineStr">
+      <c r="U16" s="14" t="inlineStr">
         <is>
           <t>#mabradiante #metas #leydeatraccion #decreto #mty</t>
         </is>
       </c>
-      <c r="Q16" s="14" t="inlineStr">
+      <c r="V16" s="14" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R16" s="14" t="inlineStr">
+      <c r="W16" s="14" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S16" s="14" t="inlineStr">
+      <c r="X16" s="14" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T16" s="14" t="inlineStr">
+      <c r="Y16" s="14" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U16" s="7" t="inlineStr"/>
-      <c r="V16" s="7" t="inlineStr"/>
-      <c r="W16" s="7" t="inlineStr"/>
-      <c r="X16" s="7" t="inlineStr"/>
-      <c r="Y16" s="7" t="inlineStr"/>
+      <c r="AA16" s="14" t="inlineStr">
+        <is>
+          <t>Pieza de venta del día (1 de 3). Vende el Nivel 1, que ya está completo.</t>
+        </is>
+      </c>
+      <c r="AB16" s="7" t="inlineStr"/>
+      <c r="AC16" s="7" t="inlineStr"/>
+      <c r="AD16" s="7" t="inlineStr"/>
+      <c r="AE16" s="7" t="inlineStr"/>
+      <c r="AF16" s="7" t="inlineStr"/>
+      <c r="AG16" s="7" t="inlineStr"/>
+      <c r="AH16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="330" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -2596,32 +3368,47 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>DOM-1</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Detecta tu programa en 2 minutos</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Domingo 11 · Pieza 1 · Patrones · el programa que se repite</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
-        <is>
-          <t>DOM-1</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>Patrones · el programa que se repite</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>G3 · Técnica paso a paso</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="K17" s="16" t="inlineStr">
         <is>
           <t>s/d</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
+      <c r="L17" s="16" t="inlineStr">
         <is>
           <t>[0:00–0:07] GANCHO: "Hoy te enseño a detectar en 2 minutos el programa que más se repite en tu vida."
 [0:07–0:16] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -2632,67 +3419,99 @@
 [0:54–0:58] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr">
+      <c r="M17" s="16" t="inlineStr">
         <is>
           <t>≈ 0:58 min (58 s)</t>
         </is>
       </c>
-      <c r="K17" s="16" t="inlineStr">
+      <c r="N17" s="16" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr">
+      <c r="O17" s="16" t="inlineStr">
         <is>
           <t>PROGRAMA</t>
         </is>
       </c>
-      <c r="M17" s="16" t="inlineStr">
+      <c r="P17" s="16" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N17" s="16" t="inlineStr">
+      <c r="Q17" s="16" t="inlineStr">
         <is>
           <t>Detecta en 2 minutos el programa que más se repite en tu vida 🧩 Guárdalo. Comenta PROGRAMA 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O17" s="16" t="inlineStr">
+      <c r="R17" s="16" t="inlineStr">
+        <is>
+          <t>Detecta en 2 minutos el programa que más se repite en tu vida 🧩 Guárdalo. Comenta PROGRAMA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S17" s="16" t="inlineStr">
+        <is>
+          <t>Detecta en 2 minutos el programa que más se repite en tu vida 🧩 Guárdalo. Comenta PROGRAMA 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T17" s="16" t="inlineStr">
         <is>
           <t>Detecta tu programa en 2 minutos #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P17" s="16" t="inlineStr">
+      <c r="U17" s="16" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q17" s="16" t="inlineStr">
+      <c r="V17" s="16" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R17" s="16" t="inlineStr">
+      <c r="W17" s="16" t="inlineStr">
         <is>
           <t>G3 · Técnica paso a paso</t>
         </is>
       </c>
-      <c r="S17" s="16" t="inlineStr">
+      <c r="X17" s="16" t="inlineStr">
         <is>
           <t>Pieza 1 abre el tema del día (rompe una creencia). Mediodía: tus TikToks de 10 a 13 h rinden 1.6x tu mediana (5 videos).</t>
         </is>
       </c>
-      <c r="T17" s="16" t="inlineStr">
+      <c r="Y17" s="16" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z17" s="16" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U17" s="7" t="inlineStr"/>
-      <c r="V17" s="7" t="inlineStr"/>
-      <c r="W17" s="7" t="inlineStr"/>
-      <c r="X17" s="7" t="inlineStr"/>
-      <c r="Y17" s="7" t="inlineStr"/>
+      <c r="AA17" s="16" t="inlineStr">
+        <is>
+          <t>Sin venta.</t>
+        </is>
+      </c>
+      <c r="AB17" s="7" t="inlineStr"/>
+      <c r="AC17" s="7" t="inlineStr"/>
+      <c r="AD17" s="7" t="inlineStr"/>
+      <c r="AE17" s="7" t="inlineStr"/>
+      <c r="AF17" s="7" t="inlineStr"/>
+      <c r="AG17" s="7" t="inlineStr"/>
+      <c r="AH17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="330" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
@@ -2710,32 +3529,47 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>DOM-2</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Espiritualidad y ciencia no son lo mismo</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Domingo 11 · Pieza 2 · Posicionamiento · espiritualidad vs ciencia</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>DOM-2</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>Posicionamiento · espiritualidad vs ciencia</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>G1 · Frase polémica</t>
         </is>
       </c>
-      <c r="H18" s="16" t="inlineStr">
+      <c r="K18" s="16" t="inlineStr">
         <is>
           <t>Sorpresa: "nunca lo había visto así"</t>
         </is>
       </c>
-      <c r="I18" s="16" t="inlineStr">
+      <c r="L18" s="16" t="inlineStr">
         <is>
           <t>[0:00–0:06] GANCHO: "No quiero convencerte de que la espiritualidad es ciencia. Quiero que aprendas a distinguirlas."
 [0:06–0:15] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -2746,67 +3580,99 @@
 [0:57–1:01] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J18" s="16" t="inlineStr">
+      <c r="M18" s="16" t="inlineStr">
         <is>
           <t>≈ 1:01 min (61 s)</t>
         </is>
       </c>
-      <c r="K18" s="16" t="inlineStr">
+      <c r="N18" s="16" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L18" s="16" t="inlineStr">
+      <c r="O18" s="16" t="inlineStr">
         <is>
           <t>MAPAS</t>
         </is>
       </c>
-      <c r="M18" s="16" t="inlineStr">
+      <c r="P18" s="16" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N18" s="16" t="inlineStr">
+      <c r="Q18" s="16" t="inlineStr">
         <is>
           <t>No quiero convencerte de que la espiritualidad es ciencia ⚖️ Guárdalo y compártelo. Comenta MAPAS 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O18" s="16" t="inlineStr">
+      <c r="R18" s="16" t="inlineStr">
+        <is>
+          <t>No quiero convencerte de que la espiritualidad es ciencia ⚖️ Guárdalo y compártelo. Comenta MAPAS 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S18" s="16" t="inlineStr">
+        <is>
+          <t>No quiero convencerte de que la espiritualidad es ciencia ⚖️ Guárdalo y compártelo. Comenta MAPAS 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T18" s="16" t="inlineStr">
         <is>
           <t>Espiritualidad y ciencia no son lo mismo #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P18" s="16" t="inlineStr">
+      <c r="U18" s="16" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q18" s="16" t="inlineStr">
+      <c r="V18" s="16" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R18" s="16" t="inlineStr">
+      <c r="W18" s="16" t="inlineStr">
         <is>
           <t>Romper creencia: "No es que… es que…" (el gancho más repetido en los virales)</t>
         </is>
       </c>
-      <c r="S18" s="16" t="inlineStr">
+      <c r="X18" s="16" t="inlineStr">
         <is>
           <t>Pieza 2 es la herramienta, la más compartible. Tu mejor horario: de 18 a 21 h tus TikToks rinden 6.3x tu mediana (7 videos).</t>
         </is>
       </c>
-      <c r="T18" s="16" t="inlineStr">
+      <c r="Y18" s="16" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 1/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 9/10</t>
+        </is>
+      </c>
+      <c r="Z18" s="16" t="inlineStr">
         <is>
           <t>9/10</t>
         </is>
       </c>
-      <c r="U18" s="7" t="inlineStr"/>
-      <c r="V18" s="7" t="inlineStr"/>
-      <c r="W18" s="7" t="inlineStr"/>
-      <c r="X18" s="7" t="inlineStr"/>
-      <c r="Y18" s="7" t="inlineStr"/>
+      <c r="AA18" s="16" t="inlineStr">
+        <is>
+          <t>Sin venta. Posiciona a Mabel con la audiencia avanzada. La microherramienta es una pregunta: vale 1 de 2.</t>
+        </is>
+      </c>
+      <c r="AB18" s="7" t="inlineStr"/>
+      <c r="AC18" s="7" t="inlineStr"/>
+      <c r="AD18" s="7" t="inlineStr"/>
+      <c r="AE18" s="7" t="inlineStr"/>
+      <c r="AF18" s="7" t="inlineStr"/>
+      <c r="AG18" s="7" t="inlineStr"/>
+      <c r="AH18" s="7" t="inlineStr"/>
     </row>
     <row r="19" ht="330" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -2824,32 +3690,47 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>DOM-3</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Decreto de domingo para tu semana</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Domingo 11 · Pieza 3 · Semana nueva · decreto</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>TikTok · Instagram Reels · Facebook Reels · YouTube Shorts</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
-        <is>
-          <t>DOM-3</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>Semana nueva · decreto</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
         <is>
           <t>G2 · Promesa práctica</t>
         </is>
       </c>
-      <c r="H19" s="16" t="inlineStr">
+      <c r="K19" s="16" t="inlineStr">
         <is>
           <t>Alivio: "algo que puedo hacer ya"</t>
         </is>
       </c>
-      <c r="I19" s="16" t="inlineStr">
+      <c r="L19" s="16" t="inlineStr">
         <is>
           <t>[0:00–0:06] GANCHO: "Di esto el domingo en la noche y empieza tu semana en otra frecuencia."
 [0:06–0:15] GUARDAR Y COMPARTIR: "Guarda este video antes de que se te pierda y compártelo con alguien que ya está lista para salir de la Matrix."
@@ -2860,94 +3741,126 @@
 [0:57–1:01] CTA: "Sígueme para más hackeos de tu mente y la Matrix."</t>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr">
+      <c r="M19" s="16" t="inlineStr">
         <is>
           <t>≈ 1:01 min (61 s)</t>
         </is>
       </c>
-      <c r="K19" s="16" t="inlineStr">
+      <c r="N19" s="16" t="inlineStr">
         <is>
           <t>Video vertical 9:16, cara a cámara. El mismo video va a las 4 redes.</t>
         </is>
       </c>
-      <c r="L19" s="16" t="inlineStr">
+      <c r="O19" s="16" t="inlineStr">
         <is>
           <t>HECHO ESTÁ</t>
         </is>
       </c>
-      <c r="M19" s="16" t="inlineStr">
+      <c r="P19" s="16" t="inlineStr">
         <is>
           <t>Sin venta (conexión)</t>
         </is>
       </c>
-      <c r="N19" s="16" t="inlineStr">
+      <c r="Q19" s="16" t="inlineStr">
         <is>
           <t>Di esto el domingo en la noche 🌙 Guárdalo para cada semana. Comenta HECHO ESTÁ 👇
 #mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="O19" s="16" t="inlineStr">
+      <c r="R19" s="16" t="inlineStr">
+        <is>
+          <t>Di esto el domingo en la noche 🌙 Guárdalo para cada semana. Comenta HECHO ESTÁ 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="S19" s="16" t="inlineStr">
+        <is>
+          <t>Di esto el domingo en la noche 🌙 Guárdalo para cada semana. Comenta HECHO ESTÁ 👇
+#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
+        </is>
+      </c>
+      <c r="T19" s="16" t="inlineStr">
         <is>
           <t>Decreto de domingo para tu semana #mabradiante #hackeatumente #espiritualidad #decreto #mty #shorts</t>
         </is>
       </c>
-      <c r="P19" s="16" t="inlineStr">
+      <c r="U19" s="16" t="inlineStr">
         <is>
           <t>#mabradiante #hackeatumente #espiritualidad #decreto #mty</t>
         </is>
       </c>
-      <c r="Q19" s="16" t="inlineStr">
+      <c r="V19" s="16" t="inlineStr">
         <is>
           <t>Meta: superar tu mediana de TikTok (11,850 vistas). Viral para ti: más de 17,775 (1.5x). Instagram, Facebook y YouTube: s/d, los medimos en la rutina semanal.</t>
         </is>
       </c>
-      <c r="R19" s="16" t="inlineStr">
+      <c r="W19" s="16" t="inlineStr">
         <is>
           <t>Algo para usar ya: decreto, respiración o ritual (tu viral de 2.2M y tus 4 más vistos)</t>
         </is>
       </c>
-      <c r="S19" s="16" t="inlineStr">
+      <c r="X19" s="16" t="inlineStr">
         <is>
           <t>Pieza 3 cierra con la venta, cuando ya calentaste el tema con las 2 anteriores. Sigue en tu mejor franja (18 a 21 h).</t>
         </is>
       </c>
-      <c r="T19" s="16" t="inlineStr">
+      <c r="Y19" s="16" t="inlineStr">
+        <is>
+          <t>Primera frase = gancho G1 a G4: 2/2
+Quita la culpa antes de enseñar: 1/1
+Un dato de ciencia simple: 1/1
+Algo para usar ya: 2/2
+Pide guardar/compartir en 15 s: 1/1
+Pide comentar una palabra: 1/1
+Venta al final en 1 frase (o sin venta): 1/1
+Vocabulario BNQ™, nada prohibido: 1/1
+Total: 10/10</t>
+        </is>
+      </c>
+      <c r="Z19" s="16" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="U19" s="7" t="inlineStr"/>
-      <c r="V19" s="7" t="inlineStr"/>
-      <c r="W19" s="7" t="inlineStr"/>
-      <c r="X19" s="7" t="inlineStr"/>
-      <c r="Y19" s="7" t="inlineStr"/>
+      <c r="AA19" s="16" t="inlineStr">
+        <is>
+          <t>Sin venta. Mismo formato que tu video viral de 2.2M.</t>
+        </is>
+      </c>
+      <c r="AB19" s="7" t="inlineStr"/>
+      <c r="AC19" s="7" t="inlineStr"/>
+      <c r="AD19" s="7" t="inlineStr"/>
+      <c r="AE19" s="7" t="inlineStr"/>
+      <c r="AF19" s="7" t="inlineStr"/>
+      <c r="AG19" s="7" t="inlineStr"/>
+      <c r="AH19" s="7" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="T21" s="18" t="inlineStr">
+      <c r="AA21" s="18" t="inlineStr">
         <is>
           <t>Grabadas:</t>
         </is>
       </c>
-      <c r="U21" s="18">
-        <f>COUNTIF(U2:U19,"Sí")&amp;" de "&amp;COUNTA(E2:E19)</f>
+      <c r="AB21" s="18">
+        <f>COUNTIF(AB2:AB19,"Sí")&amp;" de "&amp;COUNTA(D2:D19)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="T22" s="18" t="inlineStr">
+      <c r="AA22" s="18" t="inlineStr">
         <is>
           <t>Publicadas:</t>
         </is>
       </c>
-      <c r="U22" s="18">
-        <f>COUNTIF(V2:V19,"Sí")&amp;" de "&amp;COUNTA(E2:E19)</f>
+      <c r="AB22" s="18">
+        <f>COUNTIF(AC2:AC19,"Sí")&amp;" de "&amp;COUNTA(D2:D19)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y19"/>
+  <autoFilter ref="A1:AH19"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2:V19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AB2:AC19 AH2:AH19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2956,6 +3869,1020 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>PIEZA</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>TÍTULO DEL VIDEO</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>HOOK (primera frase, sin saludar)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>GUARDA (antes del segundo 15)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>PROBLEMA Y SÍNTOMA</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>REENCUADRE</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>PUENTE ESPIRITUAL + CIENTÍFICO</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>MICROHERRAMIENTA (para hacer ya)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>REVELACIÓN</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>MAR-1</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>No era ansiedad: era una mente sin dirección</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Durante años creí que tenía ansiedad. Lo que tenía era una mente que nadie me enseñó a dirigir.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Te acuestas y tu cabeza empieza a repasar todo: lo que dijiste, lo que falta, lo que podría salir mal.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>No estás rota. Tu mente está haciendo su trabajo: protegerte. Yo vivo con TDAH y aprendí que mi mente no necesitaba callarse; necesitaba dirección.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>En las tradiciones contemplativas a esto se le llama 'la mente de mono'. La psicología le llama rumiación: el cerebro repite lo que siente sin resolver.</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Esta noche escribe en un papel TODO lo que tu mente está cargando. Al final escribe: 'Por hoy, esto ya está fuera de mí.'</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Tu mente no se calma cuando la obligas. Se calma cuando siente que ya no tiene que cargarlo todo sola.</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Comenta MENTE y te mando el siguiente hackeo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>MAR-2</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Respiración de 60 segundos para la ansiedad</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Haz esto 60 segundos cuando sientas que la ansiedad te sube al pecho.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>El corazón se acelera, la respiración se corta y sientes que algo malo va a pasar aunque no esté pasando nada.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>No es debilidad: es tu sistema nervioso en modo alarma.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>La ciencia: exhalar más largo de lo que inhalas activa el sistema nervioso parasimpático, el freno natural de tu cuerpo. En mi marco BNQ™ a esto le llamo recuperar tu soberanía energética.</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Mano en el pecho. Inhala en 4… exhala en 8. Seis veces, conmigo.</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>No tienes que convencer a tu mente de que se calme. Le muestras a tu cuerpo que está a salvo y la mente lo sigue.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Guárdalo para cuando lo necesites y comenta CALMA si lo hiciste conmigo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>MAR-3</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Por qué tu mente se acelera al dormir</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>¿Por qué tu mente se acelera justo cuando por fin te acuestas a dormir?</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Todo el día corres, y en la noche, cuando todo se apaga, tu mente se prende.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>No es que no sepas descansar. Es que tu sistema nervioso aprendió que bajar la guardia es peligroso.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>La ciencia: cuando vives en estrés constante, tu cuerpo se queda en alerta y el sueño profundo cuesta más. Desde lo energético: es una mente que nunca cerró su día.</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Antes de dormir di tres veces, despacio: 'Hoy ya terminó. Mi cuerpo está a salvo.'</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>El descanso no llega cuando apagas la luz. Llega cuando tu sistema entiende que ya puede soltar.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Si tu mente no te deja dormir, en Querida Ansiedad te doy la auditoría mental y los audios para bajar su velocidad. Comenta DORMIR y te mando el link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-1</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Por qué repites la misma relación</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>No es que siempre te toque la persona equivocada. Es que tu sistema reconoce como 'amor' lo que ya conoce.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Cambias de pareja, pero la historia se repite: das de más, esperas, te decepcionas.</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>No eres tú la que está mal. Aprendiste en casa cómo se sentía el amor, y tu sistema busca lo familiar aunque duela.</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>La psicología lo explica con los estilos de apego que se forman en la infancia. En lo espiritual se habla de patrones que llegan para mostrarte lo que falta sanar.</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Escribe las 3 cosas que se repiten en TODAS tus relaciones. Ese es tu patrón, no tu destino.</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>No necesitas encontrar a otra persona. Necesitas dejar de buscar con el mismo programa.</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Comenta PATRÓN y te mando la parte 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Di esto antes de escribirle</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Di esto antes de volver a escribirle a esa persona.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Tienes el celular en la mano, sabes que no deberías, y aun así lo vas a hacer.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>No es falta de dignidad. Es tu sistema buscando alivio en lo conocido.</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>La ciencia: la incertidumbre de si te va a contestar engancha tu sistema de recompensa, por eso es tan difícil soltar el celular. En lo energético: es tu energía saliendo hacia afuera.</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Pon el celular boca abajo, respira tres veces y di: 'Me elijo a mí primero. Lo que es para mí no lo tengo que perseguir.'</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Cada vez que no escribes desde la ansiedad, le enseñas a tu cuerpo una forma nueva de amor.</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Guárdalo para la próxima vez y comenta ME ELIJO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>MIÉ-3</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Deja de esperar a que te elijan</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Si sigues esperando a que alguien te elija, este video es para ti.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Revisas si vio tu historia, si te contestó, si sigue en línea.</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>No te falta el amor de otros. Te falta una identidad que no dependa de ellos.</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>La neuroplasticidad nos dice que el cerebro aprende nuevas formas de verse a sí mismo con práctica repetida. En lo espiritual, es recordar quién eres.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Escribe cómo pensaría, hablaría y elegiría la versión de ti que ya se siente suficiente. Léelo cada mañana durante 7 días.</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Cuando cambias quién eres por dentro, cambias a quién atraes y a quién dejas ir.</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>En Crea y Activa tu Alter Ego te guío paso a paso para instalar esa identidad. Comenta ALTER EGO y te mando el link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>JUE-1</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>No estás perdida: estás despertando</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>¿Por qué ya no te hace feliz una vida que antes sí?</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Te levantas, trabajas, cumples, resuelves… y por dentro sientes que algo no encaja.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Quizá no estás perdida. Quizá estás despertando.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>En espiritualidad lo llamamos despertar de consciencia. Desde la psicología también puede ser una revisión profunda de tu identidad, tus valores y tus patrones aprendidos.</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Hazte hoy una sola pregunta: ¿qué parte de mi vida sigo sosteniendo solo porque siempre ha sido así?</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>La incomodidad no es el problema. Es la señal de que ya no cabes en la vida que construiste en automático.</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Si te pasa, comenta DESPERTANDO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>JUE-2</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>200 herramientas y ningún sistema</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Si sabes de energía, chakras, neuro y biohacking, pero sientes que todo está desconectado, escucha esto.</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Un maestro te habla del cuerpo, otro del subconsciente, otro de la energía… y terminas con 200 herramientas y ningún sistema.</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>No necesitas otra herramienta. Necesitas un mapa.</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Mi trabajo no es hacerte elegir entre espiritualidad y ciencia: es distinguir los mapas y construir el puente. La neurociencia muestra que el cerebro cambia con la repetición, no con la cantidad de información.</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Haz una lista de todas las prácticas que conoces y marca solo las que haces de verdad cada semana. Esa diferencia es tu punto de partida.</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>La transformación no está en saber más. Está en tener un orden.</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Comenta MAPA y te cuento cómo ordeno todo en mi sistema BNQ™.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>JUE-3</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>7 señales de que estás despertando</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>La primera señal de un despertar no es sentir paz. Es sentir incomodidad.</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Cuestionas lo que antes aceptabas, necesitas estar más sola, ciertas personas ya no te representan, buscas significado, empiezas a ver tus patrones, tienes preguntas nuevas y sientes que hay algo más.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Si te identificas con varias, no te estás volviendo rara: estás despertando.</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>En lo espiritual es despertar. En psicología, una etapa de revisión de identidad.</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Guarda esta lista y marca cuántas vives hoy.</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>No necesitas consumir 200 videos más para entender qué te pasa. Necesitas un primer mapa.</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Hice DESPIERTA para darte ese primer mapa. Comenta DESPIERTA y te mando el link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>VIE-1</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>No estás cansada: estás en alerta</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>No estás cansada por todo lo que haces. Estás cansada por todo lo que tu cuerpo carga en alerta.</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Duermes y despiertas cansada. Cuello tenso, mandíbula apretada, hombros arriba.</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>No es flojera. Es un sistema nervioso que no ha tenido permiso de descansar.</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>La ciencia: el estrés crónico mantiene activa la respuesta de lucha o huida, y eso agota. En lo energético: es energía que se fuga en sostenerlo todo.</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Ahora mismo: afloja la mandíbula, baja los hombros y exhala largo 3 veces. Repítelo 3 veces al día.</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Tu energía no se recupera solo durmiendo. Se recupera cuando tu cuerpo deja de defenderse.</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Comenta ENERGÍA si te pasa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>VIE-2</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Haz esto antes de tocar el celular</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Haz esto al despertar, antes de tocar el celular, y vas a sentir la diferencia en tu energía.</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Abres los ojos, agarras el celular y en un minuto ya estás respondiendo a todos menos a ti.</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>No es que te falte disciplina. Es que le entregas tu energía al mundo antes de dártela a ti.</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>La ciencia: revisar el celular apenas despiertas pone a tu cerebro en modo reacción desde el primer minuto. En mi marco BNQ™: es empezar el día sin soberanía energética.</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>1 minuto: pies en el piso, mano en el corazón, 5 respiraciones lentas y una intención: 'Hoy mi energía es mía.'</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Como empiezas tu mañana es como le enseñas a tu sistema quién manda.</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Guárdalo y comenta SOBERANA si lo haces mañana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>VIE-3</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Señales de que vives en modo supervivencia</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>¿Vives en modo supervivencia y ni siquiera te das cuenta?</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Todo te sobresalta, no puedes estar sin hacer nada y te enfermas justo cuando por fin descansas.</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Tu cuerpo no te está fallando: te está protegiendo de más.</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Biohacking es usar respiración, descanso y hábitos para hablarle a tu sistema nervioso en su idioma. La ciencia muestra que la respiración lenta ayuda a bajar la respuesta de estrés.</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Hoy pon una alarma a media tarde y haz 2 minutos de respiración lenta, sin celular.</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Salir del modo supervivencia no es hacer menos: es enseñarle a tu cuerpo que ya está a salvo.</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>En Apaga el Modo Supervivencia tienes el protocolo de biohacking para armonizar tu sistema nervioso y volver al presente. Comenta VUELVO A MÍ y te mando el link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-1</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>La meta que siempre dejas para el próximo año</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué meta llevas años diciendo 'este año sí'?</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>En enero empiezas con todo, en marzo ya lo dejaste, y en diciembre te prometes lo mismo.</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>No es falta de disciplina. Es una creencia que dice 'eso no es para mí'.</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>La psicología le llama autosabotaje: tu mente protege lo conocido, aunque no te guste. En lo espiritual: un programa que todavía no has visto.</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>Escribe tu meta y, debajo, la primera frase que aparece cuando la imaginas cumplida. Esa frase es el programa.</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>La meta no se te escapa: la frena una versión de ti que todavía no cree que la merece.</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>Comenta tu meta: este fin de semana respondo en video las que más se repitan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-2</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>1 minuto para cambiar tu frecuencia</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Hagamos esto juntas ahora: 1 minuto para cambiar tu frecuencia.</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Fin de semana, cansancio acumulado, la cabeza en mil cosas.</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>No necesitas una hora de meditación. Necesitas un minuto de coherencia.</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>La ciencia: respirar a un ritmo lento y parejo ayuda a regular tu ritmo cardiaco (coherencia cardiaca). Es la base de mi Fórmula F·01, Coherencia Energética Integral (CEI™).</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>Mano en el corazón. Inhala en 5… exhala en 5. Seis veces conmigo. Al final di: 'Estoy en coherencia.'</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
+        <is>
+          <t>Cuando tu corazón y tu mente van al mismo ritmo, todo lo demás se ordena.</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="inlineStr">
+        <is>
+          <t>Guárdalo, compártelo con alguien que necesite respirar hoy y comenta COHERENCIA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>SÁB-3</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>La creencia que no sabes que tienes</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>La creencia más peligrosa es la que no sabes que tienes.</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Haces todo 'bien', te esfuerzas, lo intentas… y algo invisible te sigue frenando.</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>No eres tú la que falla. Es un programa que aprendiste antes de poder elegirlo.</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>En espiritualidad lo llamamos programación. En psicología: aprendizaje y condicionamiento. En el Nivel 1 de Las Fórmulas Cuánticas, DESPERTAR, trabajamos los 4 estados de consciencia y el hackeo de creencias limitantes.</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>Completa esta frase sin pensar: 'Las personas como yo no pueden…'. Lo que escribas es tu creencia.</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>No puedes cambiar un programa que no ves. Verlo es el primer hackeo.</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>Si quieres hackear la creencia que no te deja avanzar, comenta NIVEL 1 y te mando el link de DESPERTAR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>DOM-1</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Detecta tu programa en 2 minutos</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Hoy te enseño a detectar en 2 minutos el programa que más se repite en tu vida.</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Cambian las personas, los trabajos y las ciudades, pero sientes lo mismo una y otra vez.</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>No es mala suerte. Es un programa que se activa siempre de la misma forma.</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>En espiritualidad: programación. En psicología: aprendizaje y condicionamiento. Distintos mapas, el mismo territorio.</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Responde 3 preguntas: ¿qué se repite? ¿qué siento cuando pasa? ¿dónde lo viví por primera vez?</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Cuando ves el programa, deja de ser destino y se vuelve una elección.</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Guárdalo para hacerlo con calma y comenta PROGRAMA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>DOM-2</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Espiritualidad y ciencia no son lo mismo</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>No quiero convencerte de que la espiritualidad es ciencia. Quiero que aprendas a distinguirlas.</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Escuchas 'está científicamente comprobado' en todos lados y ya no sabes en qué creer.</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>No tienes que elegir entre creer en todo y no creer en nada.</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>La espiritualidad tiene sus propios mapas sobre consciencia y propósito. La ciencia estudia lo que se puede medir. Mi trabajo es construir el puente sin fingir que son lo mismo.</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>La próxima vez que escuches 'está comprobado', pregúntate: ¿quién lo estudió y qué midió?</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Espiritualidad para despertar. Ciencia para comprender. Protocolos para practicar.</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>Comenta MAPAS si quieres más contenido así.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>DOM-3</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Decreto de domingo para tu semana</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Di esto el domingo en la noche y empieza tu semana en otra frecuencia.</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Guarda este video antes de que se te pierda.</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>El domingo en la noche llega la ansiedad del lunes: pendientes, cuentas, cansancio anticipado.</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>No es que odies los lunes. Es que llegas a ellos cargando la semana pasada.</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>La ciencia: tu cerebro sigue organizando lo vivido mientras duermes. En lo espiritual, un decreto es una intención dicha en voz alta.</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Antes de dormir di: 'Esta semana elijo desde quien soy ahora, no desde quien fui. Hecho está.'</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>La semana no empieza el lunes. Empieza en lo que decides esta noche.</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Guárdalo para cada domingo y comenta HECHO ESTÁ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3145,7 +5072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3459,7 +5386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>